<commit_message>
Proyecto completo final: 20 graficas, 13 hojas Excel, 9 scripts, 2 PDFs, README actualizado
</commit_message>
<xml_diff>
--- a/Logistica_Analisis_Completo.xlsx
+++ b/Logistica_Analisis_Completo.xlsx
@@ -15,6 +15,11 @@
     <sheet name="6_Analisis_ABC" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="7_Indicadores_Mensuales" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="8_Alertas_Stock" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="9_Correlaciones" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="10_Estadisticas" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="11_Varianza" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="12_Pareto_Proveedores" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="13_KPIs" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -568,6 +573,1114 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Producto</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Cant_N</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Cant_Media</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Cant_Std</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Cant_Min</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Cant_Max</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>CostoUnit_Media</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>CostoUnit_Std</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>CostoTotal_Suma</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>CostoTotal_Media</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>CostoTotal_Std</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Tiempo_Media</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Tiempo_Std</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Alimentos</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C2" t="n">
+        <v>285</v>
+      </c>
+      <c r="D2" t="n">
+        <v>147.99</v>
+      </c>
+      <c r="E2" t="n">
+        <v>58</v>
+      </c>
+      <c r="F2" t="n">
+        <v>484</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1188.78</v>
+      </c>
+      <c r="H2" t="n">
+        <v>638.78</v>
+      </c>
+      <c r="I2" t="n">
+        <v>2730460.82</v>
+      </c>
+      <c r="J2" t="n">
+        <v>390065.83</v>
+      </c>
+      <c r="K2" t="n">
+        <v>331433.54</v>
+      </c>
+      <c r="L2" t="n">
+        <v>4.14</v>
+      </c>
+      <c r="M2" t="n">
+        <v>3.08</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Electrónicos</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3" t="n">
+        <v>353.67</v>
+      </c>
+      <c r="D3" t="n">
+        <v>116.1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>245</v>
+      </c>
+      <c r="F3" t="n">
+        <v>476</v>
+      </c>
+      <c r="G3" t="n">
+        <v>713.0700000000001</v>
+      </c>
+      <c r="H3" t="n">
+        <v>650.76</v>
+      </c>
+      <c r="I3" t="n">
+        <v>849311.15</v>
+      </c>
+      <c r="J3" t="n">
+        <v>283103.72</v>
+      </c>
+      <c r="K3" t="n">
+        <v>330075.27</v>
+      </c>
+      <c r="L3" t="n">
+        <v>3</v>
+      </c>
+      <c r="M3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Farmacéuticos</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C4" t="n">
+        <v>134.5</v>
+      </c>
+      <c r="D4" t="n">
+        <v>102.84</v>
+      </c>
+      <c r="E4" t="n">
+        <v>31</v>
+      </c>
+      <c r="F4" t="n">
+        <v>267</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1185.1</v>
+      </c>
+      <c r="H4" t="n">
+        <v>604.0599999999999</v>
+      </c>
+      <c r="I4" t="n">
+        <v>459981.16</v>
+      </c>
+      <c r="J4" t="n">
+        <v>114995.29</v>
+      </c>
+      <c r="K4" t="n">
+        <v>58712.61</v>
+      </c>
+      <c r="L4" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="M4" t="n">
+        <v>5.56</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Herramientas</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>5</v>
+      </c>
+      <c r="C5" t="n">
+        <v>229.6</v>
+      </c>
+      <c r="D5" t="n">
+        <v>169.64</v>
+      </c>
+      <c r="E5" t="n">
+        <v>30</v>
+      </c>
+      <c r="F5" t="n">
+        <v>423</v>
+      </c>
+      <c r="G5" t="n">
+        <v>891.89</v>
+      </c>
+      <c r="H5" t="n">
+        <v>631.6</v>
+      </c>
+      <c r="I5" t="n">
+        <v>721165.45</v>
+      </c>
+      <c r="J5" t="n">
+        <v>144233.09</v>
+      </c>
+      <c r="K5" t="n">
+        <v>99551.84</v>
+      </c>
+      <c r="L5" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="M5" t="n">
+        <v>3.71</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Muebles</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>7</v>
+      </c>
+      <c r="C6" t="n">
+        <v>284.14</v>
+      </c>
+      <c r="D6" t="n">
+        <v>133.98</v>
+      </c>
+      <c r="E6" t="n">
+        <v>112</v>
+      </c>
+      <c r="F6" t="n">
+        <v>469</v>
+      </c>
+      <c r="G6" t="n">
+        <v>868.75</v>
+      </c>
+      <c r="H6" t="n">
+        <v>302.25</v>
+      </c>
+      <c r="I6" t="n">
+        <v>1616726.65</v>
+      </c>
+      <c r="J6" t="n">
+        <v>230960.95</v>
+      </c>
+      <c r="K6" t="n">
+        <v>117221.23</v>
+      </c>
+      <c r="L6" t="n">
+        <v>5.86</v>
+      </c>
+      <c r="M6" t="n">
+        <v>4.34</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Papelería</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>4</v>
+      </c>
+      <c r="C7" t="n">
+        <v>232.5</v>
+      </c>
+      <c r="D7" t="n">
+        <v>157.88</v>
+      </c>
+      <c r="E7" t="n">
+        <v>131</v>
+      </c>
+      <c r="F7" t="n">
+        <v>468</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1456.66</v>
+      </c>
+      <c r="H7" t="n">
+        <v>630.1799999999999</v>
+      </c>
+      <c r="I7" t="n">
+        <v>1480911.2</v>
+      </c>
+      <c r="J7" t="n">
+        <v>370227.8</v>
+      </c>
+      <c r="K7" t="n">
+        <v>352527.06</v>
+      </c>
+      <c r="L7" t="n">
+        <v>8.75</v>
+      </c>
+      <c r="M7" t="n">
+        <v>4.57</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Químicos</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>6</v>
+      </c>
+      <c r="C8" t="n">
+        <v>236.67</v>
+      </c>
+      <c r="D8" t="n">
+        <v>145.12</v>
+      </c>
+      <c r="E8" t="n">
+        <v>68</v>
+      </c>
+      <c r="F8" t="n">
+        <v>453</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1097.31</v>
+      </c>
+      <c r="H8" t="n">
+        <v>593.74</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1472806.65</v>
+      </c>
+      <c r="J8" t="n">
+        <v>245467.78</v>
+      </c>
+      <c r="K8" t="n">
+        <v>222876.54</v>
+      </c>
+      <c r="L8" t="n">
+        <v>5.33</v>
+      </c>
+      <c r="M8" t="n">
+        <v>4.37</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Ropa</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>4</v>
+      </c>
+      <c r="C9" t="n">
+        <v>292.5</v>
+      </c>
+      <c r="D9" t="n">
+        <v>143.34</v>
+      </c>
+      <c r="E9" t="n">
+        <v>109</v>
+      </c>
+      <c r="F9" t="n">
+        <v>445</v>
+      </c>
+      <c r="G9" t="n">
+        <v>713.17</v>
+      </c>
+      <c r="H9" t="n">
+        <v>706.79</v>
+      </c>
+      <c r="I9" t="n">
+        <v>867730.3100000001</v>
+      </c>
+      <c r="J9" t="n">
+        <v>216932.58</v>
+      </c>
+      <c r="K9" t="n">
+        <v>210599.83</v>
+      </c>
+      <c r="L9" t="n">
+        <v>10.75</v>
+      </c>
+      <c r="M9" t="n">
+        <v>2.06</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Suma_Total</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Desv_Estandar</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Minimo</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Maximo</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Cancelado</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C2" t="n">
+        <v>575197.87</v>
+      </c>
+      <c r="D2" t="n">
+        <v>191732.62</v>
+      </c>
+      <c r="E2" t="n">
+        <v>6436.32</v>
+      </c>
+      <c r="F2" t="n">
+        <v>184588.56</v>
+      </c>
+      <c r="G2" t="n">
+        <v>197078.91</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Devuelto</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="n">
+        <v>428810.2</v>
+      </c>
+      <c r="D3" t="n">
+        <v>214405.1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>103680.38</v>
+      </c>
+      <c r="F3" t="n">
+        <v>141092</v>
+      </c>
+      <c r="G3" t="n">
+        <v>287718.2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>En tránsito</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>12</v>
+      </c>
+      <c r="C4" t="n">
+        <v>3201650.48</v>
+      </c>
+      <c r="D4" t="n">
+        <v>266804.21</v>
+      </c>
+      <c r="E4" t="n">
+        <v>221264.96</v>
+      </c>
+      <c r="F4" t="n">
+        <v>8843.17</v>
+      </c>
+      <c r="G4" t="n">
+        <v>697677.5600000001</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Entregado</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>21</v>
+      </c>
+      <c r="C5" t="n">
+        <v>5252466.54</v>
+      </c>
+      <c r="D5" t="n">
+        <v>250117.45</v>
+      </c>
+      <c r="E5" t="n">
+        <v>273422.62</v>
+      </c>
+      <c r="F5" t="n">
+        <v>25795.8</v>
+      </c>
+      <c r="G5" t="n">
+        <v>931356.36</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" t="n">
+        <v>740968.3</v>
+      </c>
+      <c r="D6" t="n">
+        <v>370484.15</v>
+      </c>
+      <c r="E6" t="n">
+        <v>90917.28999999999</v>
+      </c>
+      <c r="F6" t="n">
+        <v>306195.92</v>
+      </c>
+      <c r="G6" t="n">
+        <v>434772.38</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Proveedor</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Costo_Total</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>%_del_Total</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>%_Acumulado</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Clasificacion</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Suministros del Sur</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>2265736.19</v>
+      </c>
+      <c r="C2" t="n">
+        <v>22.22</v>
+      </c>
+      <c r="D2" t="n">
+        <v>22.22</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>A - Vital (80% del valor)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CargoExpress</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1387386.09</v>
+      </c>
+      <c r="C3" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="D3" t="n">
+        <v>35.82</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>A - Vital (80% del valor)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>LogiTrans MX</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1230476.47</v>
+      </c>
+      <c r="C4" t="n">
+        <v>12.06</v>
+      </c>
+      <c r="D4" t="n">
+        <v>47.88</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>A - Vital (80% del valor)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>FastDelivery</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1109156.54</v>
+      </c>
+      <c r="C5" t="n">
+        <v>10.88</v>
+      </c>
+      <c r="D5" t="n">
+        <v>58.76</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>A - Vital (80% del valor)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Soluciones Logísticas</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1027378.63</v>
+      </c>
+      <c r="C6" t="n">
+        <v>10.07</v>
+      </c>
+      <c r="D6" t="n">
+        <v>68.83</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>A - Vital (80% del valor)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Distribuidora Norte</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>867316.1499999999</v>
+      </c>
+      <c r="C7" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="D7" t="n">
+        <v>77.33</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>A - Vital (80% del valor)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>MercaGlobal</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>807216.0900000001</v>
+      </c>
+      <c r="C8" t="n">
+        <v>7.91</v>
+      </c>
+      <c r="D8" t="n">
+        <v>85.23999999999999</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>B - Importante (15% del valor)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Transportes del Valle</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>508641.98</v>
+      </c>
+      <c r="C9" t="n">
+        <v>4.99</v>
+      </c>
+      <c r="D9" t="n">
+        <v>90.23</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>B - Importante (15% del valor)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ExportaTodo</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>499726.3199999999</v>
+      </c>
+      <c r="C10" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="D10" t="n">
+        <v>95.13</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>C - Complementario (5% del valor)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Importadora Central</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>496058.93</v>
+      </c>
+      <c r="C11" t="n">
+        <v>4.86</v>
+      </c>
+      <c r="D11" t="n">
+        <v>99.98999999999999</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>C - Complementario (5% del valor)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Indicador</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Valor_Actual</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>OTIF (On Time In Full)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>52.5%</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>≥ 85%</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>⚠️ Alerta</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Costo por Orden Promedio</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>$254,977.33</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>≤ $150,000</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>⚠️ Alerta</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Costo Envio por Orden</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>$3,697.01</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>≤ $1,000</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>⚠️ Alerta</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Productividad Transportista</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>3.0 envios/transp</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>≥ 15 envios</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>⚠️ Alerta</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Tiempo Promedio Entrega</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>6.5 dias</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>≤ 7 dias</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>✅ OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Satisfaccion Cliente</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>4.36/5.0</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>≥ 4.5</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>⚠️ Alerta</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Tasa Entrega Exitosa</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>52.5%</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>≥ 80%</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>⚠️ Alerta</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Total Ordenes</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Total Envios</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Valor Inventario</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>$86,097,243.77</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -3161,4 +4274,121 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Costo_Unitario</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Costo_Total</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Tiempo_Entrega_Días</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>-0.098</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.672</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-0.011</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Costo_Unitario</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>-0.098</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.582</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-0.125</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Costo_Total</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.672</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.582</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-0.093</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Tiempo_Entrega_Días</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>-0.011</v>
+      </c>
+      <c r="C5" t="n">
+        <v>-0.125</v>
+      </c>
+      <c r="D5" t="n">
+        <v>-0.093</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>